<commit_message>
Updates to the code writing Excel reports - mainly to improve the headers.
</commit_message>
<xml_diff>
--- a/inst/extdata/Report - column names - no replicates.xlsx
+++ b/inst/extdata/Report - column names - no replicates.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\aRmel package\aRmel\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\home\aRmel_package\proteoCraft\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11C83C31-C4AE-4B70-A787-61738C9B81D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="12735" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="1" r:id="rId1"/>
@@ -20,12 +21,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="136">
   <si>
     <t>Columns:</t>
   </si>
@@ -460,9 +464,6 @@
     <t>Analysis run by:</t>
   </si>
   <si>
-    <t>For protein groups/peptidoforms matching proteins of interest, text is coloured brick red.</t>
-  </si>
-  <si>
     <t>Package version:</t>
   </si>
   <si>
@@ -827,8 +828,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="30" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -927,14 +928,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FFA52A2A"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -1510,7 +1503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="156">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1602,9 +1595,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1621,7 +1611,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1642,7 +1632,7 @@
     <xf numFmtId="3" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1657,13 +1647,13 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="19" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="18" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1672,7 +1662,7 @@
     <xf numFmtId="3" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1681,10 +1671,10 @@
     <xf numFmtId="3" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="19" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="18" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1693,10 +1683,10 @@
     <xf numFmtId="3" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="19" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="18" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1705,7 +1695,7 @@
     <xf numFmtId="3" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1714,10 +1704,10 @@
     <xf numFmtId="3" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="19" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="18" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1726,7 +1716,7 @@
     <xf numFmtId="3" fontId="1" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1753,27 +1743,27 @@
     <xf numFmtId="49" fontId="1" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="20" fillId="38" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="21" fillId="38" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="38" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1820,6 +1810,27 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1847,41 +1858,50 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="41" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="41" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="42" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1892,9 +1912,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1904,6 +1921,15 @@
     <xf numFmtId="0" fontId="0" fillId="40" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1921,42 +1947,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="42" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2237,8 +2227,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P57"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:P55"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -2263,88 +2253,88 @@
       <c r="I1" s="31"/>
       <c r="J1" s="31"/>
       <c r="K1" s="31"/>
-      <c r="L1" s="97"/>
-      <c r="M1" s="97"/>
+      <c r="L1" s="96"/>
+      <c r="M1" s="96"/>
       <c r="N1" s="32"/>
       <c r="O1" s="25"/>
       <c r="P1" s="25"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="25"/>
-      <c r="B2" s="40" t="s">
-        <v>81</v>
+      <c r="B2" s="39" t="s">
+        <v>80</v>
       </c>
       <c r="C2" s="27"/>
       <c r="D2" s="25"/>
-      <c r="E2" s="42"/>
+      <c r="E2" s="41"/>
       <c r="F2" s="31"/>
       <c r="G2" s="31"/>
       <c r="H2" s="31"/>
       <c r="I2" s="31"/>
       <c r="J2" s="31"/>
       <c r="K2" s="31"/>
-      <c r="L2" s="97"/>
-      <c r="M2" s="97"/>
+      <c r="L2" s="96"/>
+      <c r="M2" s="96"/>
       <c r="N2" s="32"/>
       <c r="O2" s="25"/>
       <c r="P2" s="25"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="25"/>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="39" t="s">
         <v>77</v>
       </c>
       <c r="C3" s="27"/>
       <c r="D3" s="25"/>
-      <c r="E3" s="42"/>
+      <c r="E3" s="41"/>
       <c r="F3" s="31"/>
       <c r="G3" s="31"/>
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
       <c r="J3" s="31"/>
       <c r="K3" s="31"/>
-      <c r="L3" s="97"/>
-      <c r="M3" s="97"/>
+      <c r="L3" s="96"/>
+      <c r="M3" s="96"/>
       <c r="N3" s="32"/>
       <c r="O3" s="25"/>
       <c r="P3" s="25"/>
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="25"/>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="39" t="s">
         <v>78</v>
       </c>
       <c r="C4" s="27"/>
       <c r="D4" s="25"/>
-      <c r="E4" s="42"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="31"/>
       <c r="G4" s="31"/>
       <c r="H4" s="31"/>
       <c r="I4" s="31"/>
       <c r="J4" s="31"/>
       <c r="K4" s="31"/>
-      <c r="L4" s="97"/>
-      <c r="M4" s="97"/>
+      <c r="L4" s="96"/>
+      <c r="M4" s="96"/>
       <c r="N4" s="32"/>
       <c r="O4" s="25"/>
       <c r="P4" s="25"/>
     </row>
     <row r="5" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="25"/>
-      <c r="B5" s="40" t="s">
-        <v>80</v>
+      <c r="B5" s="39" t="s">
+        <v>79</v>
       </c>
       <c r="C5" s="27"/>
       <c r="D5" s="25"/>
-      <c r="E5" s="42"/>
+      <c r="E5" s="41"/>
       <c r="F5" s="31"/>
       <c r="G5" s="31"/>
       <c r="H5" s="31"/>
       <c r="I5" s="31"/>
       <c r="J5" s="31"/>
       <c r="K5" s="31"/>
-      <c r="L5" s="97"/>
-      <c r="M5" s="97"/>
+      <c r="L5" s="96"/>
+      <c r="M5" s="96"/>
       <c r="N5" s="32"/>
       <c r="O5" s="25"/>
       <c r="P5" s="25"/>
@@ -2361,205 +2351,215 @@
       <c r="I6" s="31"/>
       <c r="J6" s="31"/>
       <c r="K6" s="31"/>
-      <c r="L6" s="97"/>
-      <c r="M6" s="97"/>
+      <c r="L6" s="96"/>
+      <c r="M6" s="96"/>
       <c r="N6" s="32"/>
       <c r="O6" s="25"/>
       <c r="P6" s="25"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="25"/>
-      <c r="B7" s="33" t="s">
-        <v>79</v>
-      </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="29"/>
+      <c r="B7" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="27"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="33"/>
       <c r="F7" s="31"/>
       <c r="G7" s="31"/>
       <c r="H7" s="31"/>
       <c r="I7" s="31"/>
-      <c r="J7" s="31"/>
-      <c r="K7" s="31"/>
-      <c r="L7" s="99"/>
-      <c r="M7" s="99"/>
-      <c r="N7" s="99"/>
-      <c r="O7" s="99"/>
-      <c r="P7" s="99"/>
+      <c r="J7" s="25"/>
+      <c r="K7" s="25"/>
+      <c r="L7" s="98"/>
+      <c r="M7" s="98"/>
+      <c r="N7" s="98"/>
+      <c r="O7" s="98"/>
+      <c r="P7" s="98"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="25"/>
-      <c r="K8" s="25"/>
-      <c r="L8" s="99"/>
-      <c r="M8" s="99"/>
-      <c r="N8" s="99"/>
-      <c r="O8" s="99"/>
-      <c r="P8" s="99"/>
+      <c r="A8" s="34"/>
+      <c r="B8" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="37"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="34"/>
+      <c r="K8" s="34"/>
+      <c r="L8" s="98"/>
+      <c r="M8" s="98"/>
+      <c r="N8" s="98"/>
+      <c r="O8" s="98"/>
+      <c r="P8" s="98"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="25"/>
-      <c r="B9" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="C9" s="27"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="34"/>
+      <c r="B9" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="33"/>
       <c r="F9" s="31"/>
       <c r="G9" s="31"/>
       <c r="H9" s="31"/>
       <c r="I9" s="31"/>
       <c r="J9" s="25"/>
       <c r="K9" s="25"/>
-      <c r="L9" s="99"/>
-      <c r="M9" s="99"/>
-      <c r="N9" s="99"/>
-      <c r="O9" s="99"/>
-      <c r="P9" s="99"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="35"/>
-      <c r="B10" s="36" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="36"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="38"/>
-      <c r="I10" s="38"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="35"/>
-      <c r="L10" s="99"/>
-      <c r="M10" s="99"/>
-      <c r="N10" s="99"/>
-      <c r="O10" s="99"/>
-      <c r="P10" s="99"/>
-    </row>
-    <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L9" s="98"/>
+      <c r="M9" s="98"/>
+      <c r="N9" s="98"/>
+      <c r="O9" s="98"/>
+      <c r="P9" s="98"/>
+    </row>
+    <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="25"/>
+      <c r="B10" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="118" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" s="118"/>
+      <c r="H10" s="118"/>
+      <c r="I10" s="118"/>
+      <c r="J10" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="K10" s="25"/>
+      <c r="L10" s="98"/>
+      <c r="M10" s="98"/>
+      <c r="N10" s="98"/>
+      <c r="O10" s="98"/>
+      <c r="P10" s="98"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="25"/>
-      <c r="B11" s="36" t="s">
-        <v>56</v>
-      </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="31"/>
-      <c r="J11" s="25"/>
+      <c r="B11" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" s="15"/>
+      <c r="E11" s="110"/>
+      <c r="F11" s="119"/>
+      <c r="G11" s="119"/>
+      <c r="H11" s="119"/>
+      <c r="I11" s="119"/>
+      <c r="J11" s="103"/>
       <c r="K11" s="25"/>
-      <c r="L11" s="99"/>
-      <c r="M11" s="99"/>
-      <c r="N11" s="99"/>
-      <c r="O11" s="99"/>
-      <c r="P11" s="99"/>
-    </row>
-    <row r="12" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L11" s="98"/>
+      <c r="M11" s="98"/>
+      <c r="N11" s="98"/>
+      <c r="O11" s="98"/>
+      <c r="P11" s="98"/>
+    </row>
+    <row r="12" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="25"/>
-      <c r="B12" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="F12" s="112" t="s">
-        <v>65</v>
-      </c>
-      <c r="G12" s="112"/>
-      <c r="H12" s="112"/>
-      <c r="I12" s="112"/>
-      <c r="J12" s="24" t="s">
-        <v>44</v>
-      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="111" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="120"/>
+      <c r="G12" s="120"/>
+      <c r="H12" s="120"/>
+      <c r="I12" s="120"/>
+      <c r="J12" s="104"/>
       <c r="K12" s="25"/>
-      <c r="L12" s="99"/>
-      <c r="M12" s="99"/>
-      <c r="N12" s="99"/>
-      <c r="O12" s="99"/>
-      <c r="P12" s="99"/>
+      <c r="L12" s="98"/>
+      <c r="M12" s="98"/>
+      <c r="N12" s="98"/>
+      <c r="O12" s="98"/>
+      <c r="P12" s="98"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="25"/>
-      <c r="B13" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="D13" s="15"/>
-      <c r="E13" s="146"/>
-      <c r="F13" s="113"/>
-      <c r="G13" s="113"/>
-      <c r="H13" s="113"/>
-      <c r="I13" s="113"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" s="111" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="120"/>
+      <c r="G13" s="120"/>
+      <c r="H13" s="120"/>
+      <c r="I13" s="120"/>
       <c r="J13" s="104"/>
       <c r="K13" s="25"/>
-      <c r="L13" s="99"/>
-      <c r="M13" s="99"/>
-      <c r="N13" s="99"/>
-      <c r="O13" s="99"/>
-      <c r="P13" s="99"/>
-    </row>
-    <row r="14" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L13" s="98"/>
+      <c r="M13" s="98"/>
+      <c r="N13" s="98"/>
+      <c r="O13" s="98"/>
+      <c r="P13" s="98"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="25"/>
       <c r="B14" s="16"/>
       <c r="C14" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="E14" s="147" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" s="114"/>
-      <c r="G14" s="114"/>
-      <c r="H14" s="114"/>
-      <c r="I14" s="114"/>
-      <c r="J14" s="105"/>
+        <v>4</v>
+      </c>
+      <c r="E14" s="111" t="s">
+        <v>5</v>
+      </c>
+      <c r="F14" s="120"/>
+      <c r="G14" s="120"/>
+      <c r="H14" s="120"/>
+      <c r="I14" s="120"/>
+      <c r="J14" s="104"/>
       <c r="K14" s="25"/>
-      <c r="L14" s="99"/>
-      <c r="M14" s="99"/>
-      <c r="N14" s="99"/>
-      <c r="O14" s="99"/>
-      <c r="P14" s="99"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L14" s="98"/>
+      <c r="M14" s="98"/>
+      <c r="N14" s="98"/>
+      <c r="O14" s="98"/>
+      <c r="P14" s="98"/>
+    </row>
+    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="25"/>
       <c r="B15" s="16"/>
       <c r="C15" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="E15" s="147" t="s">
-        <v>9</v>
-      </c>
-      <c r="F15" s="114"/>
-      <c r="G15" s="114"/>
-      <c r="H15" s="114"/>
-      <c r="I15" s="114"/>
-      <c r="J15" s="105"/>
+        <v>6</v>
+      </c>
+      <c r="E15" s="111" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="120"/>
+      <c r="G15" s="120"/>
+      <c r="H15" s="120"/>
+      <c r="I15" s="120"/>
+      <c r="J15" s="104"/>
       <c r="K15" s="25"/>
-      <c r="L15" s="99"/>
-      <c r="M15" s="99"/>
-      <c r="N15" s="99"/>
-      <c r="O15" s="99"/>
-      <c r="P15" s="99"/>
+      <c r="L15" s="98"/>
+      <c r="M15" s="98"/>
+      <c r="N15" s="98"/>
+      <c r="O15" s="98"/>
+      <c r="P15" s="98"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="25"/>
@@ -2568,494 +2568,490 @@
         <v>57</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="E16" s="147" t="s">
-        <v>5</v>
-      </c>
-      <c r="F16" s="114"/>
-      <c r="G16" s="114"/>
-      <c r="H16" s="114"/>
-      <c r="I16" s="114"/>
-      <c r="J16" s="105"/>
+        <v>7</v>
+      </c>
+      <c r="E16" s="111" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="120"/>
+      <c r="G16" s="120"/>
+      <c r="H16" s="120"/>
+      <c r="I16" s="120"/>
+      <c r="J16" s="104"/>
       <c r="K16" s="25"/>
-      <c r="L16" s="99"/>
-      <c r="M16" s="99"/>
-      <c r="N16" s="99"/>
-      <c r="O16" s="99"/>
-      <c r="P16" s="99"/>
-    </row>
-    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L16" s="98"/>
+      <c r="M16" s="98"/>
+      <c r="N16" s="98"/>
+      <c r="O16" s="98"/>
+      <c r="P16" s="98"/>
+    </row>
+    <row r="17" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="25"/>
-      <c r="B17" s="16"/>
+      <c r="B17" s="17"/>
       <c r="C17" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="E17" s="147" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17" s="114"/>
-      <c r="G17" s="114"/>
-      <c r="H17" s="114"/>
-      <c r="I17" s="114"/>
-      <c r="J17" s="105"/>
+        <v>11</v>
+      </c>
+      <c r="E17" s="111" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" s="120"/>
+      <c r="G17" s="120"/>
+      <c r="H17" s="120"/>
+      <c r="I17" s="120"/>
+      <c r="J17" s="104"/>
       <c r="K17" s="25"/>
-      <c r="L17" s="99"/>
-      <c r="M17" s="99"/>
-      <c r="N17" s="99"/>
-      <c r="O17" s="99"/>
-      <c r="P17" s="99"/>
+      <c r="L17" s="98"/>
+      <c r="M17" s="98"/>
+      <c r="N17" s="98"/>
+      <c r="O17" s="98"/>
+      <c r="P17" s="98"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="25"/>
-      <c r="B18" s="16"/>
+      <c r="B18" s="17"/>
       <c r="C18" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E18" s="147" t="s">
-        <v>8</v>
-      </c>
-      <c r="F18" s="114"/>
-      <c r="G18" s="114"/>
-      <c r="H18" s="114"/>
-      <c r="I18" s="114"/>
-      <c r="J18" s="105"/>
+      <c r="D18" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="111" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="120"/>
+      <c r="G18" s="120"/>
+      <c r="H18" s="120"/>
+      <c r="I18" s="120"/>
+      <c r="J18" s="104"/>
       <c r="K18" s="25"/>
-      <c r="L18" s="99"/>
-      <c r="M18" s="99"/>
-      <c r="N18" s="99"/>
-      <c r="O18" s="99"/>
-      <c r="P18" s="99"/>
-    </row>
-    <row r="19" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L18" s="98"/>
+      <c r="M18" s="98"/>
+      <c r="N18" s="98"/>
+      <c r="O18" s="98"/>
+      <c r="P18" s="98"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="25"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" s="147" t="s">
-        <v>70</v>
-      </c>
-      <c r="F19" s="114"/>
-      <c r="G19" s="114"/>
-      <c r="H19" s="114"/>
-      <c r="I19" s="114"/>
-      <c r="J19" s="105"/>
+      <c r="B19" s="42" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="43"/>
+      <c r="E19" s="112" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="121"/>
+      <c r="G19" s="121"/>
+      <c r="H19" s="121"/>
+      <c r="I19" s="121"/>
+      <c r="J19" s="130"/>
       <c r="K19" s="25"/>
-      <c r="L19" s="99"/>
-      <c r="M19" s="99"/>
-      <c r="N19" s="99"/>
-      <c r="O19" s="99"/>
-      <c r="P19" s="99"/>
+      <c r="L19" s="98"/>
+      <c r="M19" s="98"/>
+      <c r="N19" s="98"/>
+      <c r="O19" s="98"/>
+      <c r="P19" s="98"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="25"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="5" t="s">
+      <c r="B20" s="44"/>
+      <c r="C20" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" s="147" t="s">
-        <v>13</v>
-      </c>
-      <c r="F20" s="114"/>
-      <c r="G20" s="114"/>
-      <c r="H20" s="114"/>
-      <c r="I20" s="114"/>
-      <c r="J20" s="105"/>
+      <c r="D20" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="112" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="121"/>
+      <c r="G20" s="121"/>
+      <c r="H20" s="121"/>
+      <c r="I20" s="121"/>
+      <c r="J20" s="130"/>
       <c r="K20" s="25"/>
-      <c r="L20" s="99"/>
-      <c r="M20" s="99"/>
-      <c r="N20" s="99"/>
-      <c r="O20" s="99"/>
-      <c r="P20" s="99"/>
+      <c r="L20" s="98"/>
+      <c r="M20" s="98"/>
+      <c r="N20" s="98"/>
+      <c r="O20" s="98"/>
+      <c r="P20" s="98"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="25"/>
-      <c r="B21" s="43" t="s">
-        <v>58</v>
-      </c>
-      <c r="C21" s="44" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" s="44"/>
-      <c r="E21" s="148" t="s">
-        <v>15</v>
-      </c>
-      <c r="F21" s="115"/>
-      <c r="G21" s="115"/>
-      <c r="H21" s="115"/>
-      <c r="I21" s="115"/>
-      <c r="J21" s="123"/>
+      <c r="B21" s="44"/>
+      <c r="C21" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="D21" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="E21" s="112" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" s="121"/>
+      <c r="G21" s="121"/>
+      <c r="H21" s="121"/>
+      <c r="I21" s="121"/>
+      <c r="J21" s="130"/>
       <c r="K21" s="25"/>
-      <c r="L21" s="99"/>
-      <c r="M21" s="99"/>
-      <c r="N21" s="99"/>
-      <c r="O21" s="99"/>
-      <c r="P21" s="99"/>
+      <c r="L21" s="98"/>
+      <c r="M21" s="98"/>
+      <c r="N21" s="98"/>
+      <c r="O21" s="98"/>
+      <c r="P21" s="98"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="25"/>
-      <c r="B22" s="45"/>
-      <c r="C22" s="46" t="s">
-        <v>57</v>
-      </c>
-      <c r="D22" s="47" t="s">
-        <v>16</v>
-      </c>
-      <c r="E22" s="148" t="s">
-        <v>17</v>
-      </c>
-      <c r="F22" s="115"/>
-      <c r="G22" s="115"/>
-      <c r="H22" s="115"/>
-      <c r="I22" s="115"/>
-      <c r="J22" s="123"/>
+      <c r="B22" s="42" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="43"/>
+      <c r="E22" s="112" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="121"/>
+      <c r="G22" s="121"/>
+      <c r="H22" s="121"/>
+      <c r="I22" s="121"/>
+      <c r="J22" s="130"/>
       <c r="K22" s="25"/>
-      <c r="L22" s="99"/>
-      <c r="M22" s="99"/>
-      <c r="N22" s="99"/>
-      <c r="O22" s="99"/>
-      <c r="P22" s="99"/>
+      <c r="L22" s="98"/>
+      <c r="M22" s="98"/>
+      <c r="N22" s="98"/>
+      <c r="O22" s="98"/>
+      <c r="P22" s="98"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="25"/>
-      <c r="B23" s="45"/>
-      <c r="C23" s="46" t="s">
+      <c r="B23" s="44"/>
+      <c r="C23" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="D23" s="47" t="s">
-        <v>18</v>
-      </c>
-      <c r="E23" s="148" t="s">
-        <v>71</v>
-      </c>
-      <c r="F23" s="115"/>
-      <c r="G23" s="115"/>
-      <c r="H23" s="115"/>
-      <c r="I23" s="115"/>
-      <c r="J23" s="123"/>
+      <c r="D23" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="112" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="121"/>
+      <c r="G23" s="121"/>
+      <c r="H23" s="121"/>
+      <c r="I23" s="121"/>
+      <c r="J23" s="130"/>
       <c r="K23" s="25"/>
-      <c r="L23" s="99"/>
-      <c r="M23" s="99"/>
-      <c r="N23" s="99"/>
-      <c r="O23" s="99"/>
-      <c r="P23" s="99"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L23" s="98"/>
+      <c r="M23" s="98"/>
+      <c r="N23" s="98"/>
+      <c r="O23" s="98"/>
+      <c r="P23" s="98"/>
+    </row>
+    <row r="24" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="25"/>
-      <c r="B24" s="43" t="s">
-        <v>58</v>
-      </c>
-      <c r="C24" s="44" t="s">
-        <v>24</v>
-      </c>
-      <c r="D24" s="44"/>
-      <c r="E24" s="148" t="s">
-        <v>28</v>
-      </c>
-      <c r="F24" s="115"/>
-      <c r="G24" s="115"/>
-      <c r="H24" s="115"/>
-      <c r="I24" s="115"/>
-      <c r="J24" s="123"/>
+      <c r="B24" s="44"/>
+      <c r="C24" s="47" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24" s="112" t="s">
+        <v>39</v>
+      </c>
+      <c r="F24" s="121"/>
+      <c r="G24" s="121"/>
+      <c r="H24" s="121"/>
+      <c r="I24" s="121"/>
+      <c r="J24" s="130"/>
       <c r="K24" s="25"/>
-      <c r="L24" s="99"/>
-      <c r="M24" s="99"/>
-      <c r="N24" s="99"/>
-      <c r="O24" s="99"/>
-      <c r="P24" s="99"/>
+      <c r="L24" s="98"/>
+      <c r="M24" s="98"/>
+      <c r="N24" s="98"/>
+      <c r="O24" s="98"/>
+      <c r="P24" s="98"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="25"/>
-      <c r="B25" s="45"/>
-      <c r="C25" s="48" t="s">
+      <c r="B25" s="44"/>
+      <c r="C25" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="D25" s="47" t="s">
-        <v>16</v>
-      </c>
-      <c r="E25" s="148" t="s">
-        <v>40</v>
-      </c>
-      <c r="F25" s="115"/>
-      <c r="G25" s="115"/>
-      <c r="H25" s="115"/>
-      <c r="I25" s="115"/>
-      <c r="J25" s="123"/>
+      <c r="D25" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="112" t="s">
+        <v>38</v>
+      </c>
+      <c r="F25" s="121"/>
+      <c r="G25" s="121"/>
+      <c r="H25" s="121"/>
+      <c r="I25" s="121"/>
+      <c r="J25" s="130"/>
       <c r="K25" s="25"/>
-      <c r="L25" s="99"/>
-      <c r="M25" s="99"/>
-      <c r="N25" s="99"/>
-      <c r="O25" s="99"/>
-      <c r="P25" s="99"/>
-    </row>
-    <row r="26" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L25" s="98"/>
+      <c r="M25" s="98"/>
+      <c r="N25" s="98"/>
+      <c r="O25" s="98"/>
+      <c r="P25" s="98"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="25"/>
-      <c r="B26" s="45"/>
-      <c r="C26" s="48" t="s">
+      <c r="B26" s="44"/>
+      <c r="C26" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="D26" s="47" t="s">
-        <v>19</v>
-      </c>
-      <c r="E26" s="148" t="s">
-        <v>39</v>
-      </c>
-      <c r="F26" s="115"/>
-      <c r="G26" s="115"/>
-      <c r="H26" s="115"/>
-      <c r="I26" s="115"/>
-      <c r="J26" s="123"/>
+      <c r="D26" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" s="112" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" s="121"/>
+      <c r="G26" s="121"/>
+      <c r="H26" s="121"/>
+      <c r="I26" s="121"/>
+      <c r="J26" s="130"/>
       <c r="K26" s="25"/>
-      <c r="L26" s="99"/>
-      <c r="M26" s="99"/>
-      <c r="N26" s="99"/>
-      <c r="O26" s="99"/>
-      <c r="P26" s="99"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L26" s="98"/>
+      <c r="M26" s="98"/>
+      <c r="N26" s="98"/>
+      <c r="O26" s="98"/>
+      <c r="P26" s="98"/>
+    </row>
+    <row r="27" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="25"/>
-      <c r="B27" s="45"/>
-      <c r="C27" s="48" t="s">
+      <c r="B27" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D27" s="12"/>
+      <c r="E27" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" s="122"/>
+      <c r="G27" s="122"/>
+      <c r="H27" s="122"/>
+      <c r="I27" s="122"/>
+      <c r="J27" s="131"/>
+      <c r="K27" s="25"/>
+      <c r="L27" s="98"/>
+      <c r="M27" s="98"/>
+      <c r="N27" s="98"/>
+      <c r="O27" s="98"/>
+      <c r="P27" s="98"/>
+    </row>
+    <row r="28" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="25"/>
+      <c r="B28" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D28" s="12"/>
+      <c r="E28" s="126"/>
+      <c r="F28" s="122"/>
+      <c r="G28" s="122"/>
+      <c r="H28" s="122"/>
+      <c r="I28" s="122"/>
+      <c r="J28" s="131"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="98"/>
+      <c r="M28" s="98"/>
+      <c r="N28" s="98"/>
+      <c r="O28" s="98"/>
+      <c r="P28" s="98"/>
+    </row>
+    <row r="29" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="25"/>
+      <c r="B29" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="30"/>
+      <c r="E29" s="127" t="s">
+        <v>29</v>
+      </c>
+      <c r="F29" s="123"/>
+      <c r="G29" s="123"/>
+      <c r="H29" s="123"/>
+      <c r="I29" s="123"/>
+      <c r="J29" s="132"/>
+      <c r="K29" s="25"/>
+      <c r="L29" s="98"/>
+      <c r="M29" s="98"/>
+      <c r="N29" s="98"/>
+      <c r="O29" s="98"/>
+      <c r="P29" s="98"/>
+    </row>
+    <row r="30" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="25"/>
+      <c r="B30" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="D30" s="30"/>
+      <c r="E30" s="127"/>
+      <c r="F30" s="123"/>
+      <c r="G30" s="123"/>
+      <c r="H30" s="123"/>
+      <c r="I30" s="123"/>
+      <c r="J30" s="132"/>
+      <c r="K30" s="25"/>
+      <c r="L30" s="98"/>
+      <c r="M30" s="98"/>
+      <c r="N30" s="98"/>
+      <c r="O30" s="98"/>
+      <c r="P30" s="98"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="25"/>
+      <c r="B31" s="40" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" s="50"/>
+      <c r="D31" s="50"/>
+      <c r="E31" s="113"/>
+      <c r="F31" s="124"/>
+      <c r="G31" s="124"/>
+      <c r="H31" s="124"/>
+      <c r="I31" s="124"/>
+      <c r="J31" s="105"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="98"/>
+      <c r="M31" s="98"/>
+      <c r="N31" s="98"/>
+      <c r="O31" s="98"/>
+      <c r="P31" s="98"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="25"/>
+      <c r="B32" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D32" s="7"/>
+      <c r="E32" s="114"/>
+      <c r="F32" s="125"/>
+      <c r="G32" s="125"/>
+      <c r="H32" s="125"/>
+      <c r="I32" s="125"/>
+      <c r="J32" s="133" t="s">
+        <v>129</v>
+      </c>
+      <c r="K32" s="25"/>
+      <c r="L32" s="98"/>
+      <c r="M32" s="98"/>
+      <c r="N32" s="98"/>
+      <c r="O32" s="98"/>
+      <c r="P32" s="98"/>
+    </row>
+    <row r="33" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="25"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="47" t="s">
-        <v>20</v>
-      </c>
-      <c r="E27" s="148" t="s">
-        <v>38</v>
-      </c>
-      <c r="F27" s="115"/>
-      <c r="G27" s="115"/>
-      <c r="H27" s="115"/>
-      <c r="I27" s="115"/>
-      <c r="J27" s="123"/>
-      <c r="K27" s="25"/>
-      <c r="L27" s="99"/>
-      <c r="M27" s="99"/>
-      <c r="N27" s="99"/>
-      <c r="O27" s="99"/>
-      <c r="P27" s="99"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A28" s="25"/>
-      <c r="B28" s="45"/>
-      <c r="C28" s="46" t="s">
+      <c r="D33" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E33" s="114" t="s">
+        <v>72</v>
+      </c>
+      <c r="F33" s="125"/>
+      <c r="G33" s="125"/>
+      <c r="H33" s="125"/>
+      <c r="I33" s="125"/>
+      <c r="J33" s="134"/>
+      <c r="K33" s="25"/>
+      <c r="L33" s="98"/>
+      <c r="M33" s="98"/>
+      <c r="N33" s="98"/>
+      <c r="O33" s="98"/>
+      <c r="P33" s="98"/>
+    </row>
+    <row r="34" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="25"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="46" t="s">
-        <v>18</v>
-      </c>
-      <c r="E28" s="148" t="s">
-        <v>21</v>
-      </c>
-      <c r="F28" s="115"/>
-      <c r="G28" s="115"/>
-      <c r="H28" s="115"/>
-      <c r="I28" s="115"/>
-      <c r="J28" s="123"/>
-      <c r="K28" s="25"/>
-      <c r="L28" s="99"/>
-      <c r="M28" s="99"/>
-      <c r="N28" s="99"/>
-      <c r="O28" s="99"/>
-      <c r="P28" s="99"/>
-    </row>
-    <row r="29" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="25"/>
-      <c r="B29" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="D29" s="12"/>
-      <c r="E29" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="F29" s="116"/>
-      <c r="G29" s="116"/>
-      <c r="H29" s="116"/>
-      <c r="I29" s="116"/>
-      <c r="J29" s="124"/>
-      <c r="K29" s="25"/>
-      <c r="L29" s="99"/>
-      <c r="M29" s="99"/>
-      <c r="N29" s="99"/>
-      <c r="O29" s="99"/>
-      <c r="P29" s="99"/>
-    </row>
-    <row r="30" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="25"/>
-      <c r="B30" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D30" s="12"/>
-      <c r="E30" s="149"/>
-      <c r="F30" s="116"/>
-      <c r="G30" s="116"/>
-      <c r="H30" s="116"/>
-      <c r="I30" s="116"/>
-      <c r="J30" s="124"/>
-      <c r="K30" s="25"/>
-      <c r="L30" s="99"/>
-      <c r="M30" s="99"/>
-      <c r="N30" s="99"/>
-      <c r="O30" s="99"/>
-      <c r="P30" s="99"/>
-    </row>
-    <row r="31" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="25"/>
-      <c r="B31" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="C31" s="30" t="s">
-        <v>25</v>
-      </c>
-      <c r="D31" s="30"/>
-      <c r="E31" s="150" t="s">
-        <v>29</v>
-      </c>
-      <c r="F31" s="117"/>
-      <c r="G31" s="117"/>
-      <c r="H31" s="117"/>
-      <c r="I31" s="117"/>
-      <c r="J31" s="125"/>
-      <c r="K31" s="25"/>
-      <c r="L31" s="99"/>
-      <c r="M31" s="99"/>
-      <c r="N31" s="99"/>
-      <c r="O31" s="99"/>
-      <c r="P31" s="99"/>
-    </row>
-    <row r="32" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="25"/>
-      <c r="B32" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="C32" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="D32" s="30"/>
-      <c r="E32" s="150"/>
-      <c r="F32" s="117"/>
-      <c r="G32" s="117"/>
-      <c r="H32" s="117"/>
-      <c r="I32" s="117"/>
-      <c r="J32" s="125"/>
-      <c r="K32" s="25"/>
-      <c r="L32" s="99"/>
-      <c r="M32" s="99"/>
-      <c r="N32" s="99"/>
-      <c r="O32" s="99"/>
-      <c r="P32" s="99"/>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="25"/>
-      <c r="B33" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="C33" s="51"/>
-      <c r="D33" s="51"/>
-      <c r="E33" s="151"/>
-      <c r="F33" s="118"/>
-      <c r="G33" s="118"/>
-      <c r="H33" s="118"/>
-      <c r="I33" s="118"/>
-      <c r="J33" s="106"/>
-      <c r="K33" s="25"/>
-      <c r="L33" s="99"/>
-      <c r="M33" s="99"/>
-      <c r="N33" s="99"/>
-      <c r="O33" s="99"/>
-      <c r="P33" s="99"/>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A34" s="25"/>
-      <c r="B34" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D34" s="7"/>
-      <c r="E34" s="152"/>
-      <c r="F34" s="119"/>
-      <c r="G34" s="119"/>
-      <c r="H34" s="119"/>
-      <c r="I34" s="119"/>
-      <c r="J34" s="126" t="s">
-        <v>130</v>
-      </c>
+      <c r="D34" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E34" s="140" t="s">
+        <v>37</v>
+      </c>
+      <c r="F34" s="125"/>
+      <c r="G34" s="125"/>
+      <c r="H34" s="125"/>
+      <c r="I34" s="125"/>
+      <c r="J34" s="134"/>
       <c r="K34" s="25"/>
-      <c r="L34" s="99"/>
-      <c r="M34" s="99"/>
-      <c r="N34" s="99"/>
-      <c r="O34" s="99"/>
-      <c r="P34" s="99"/>
-    </row>
-    <row r="35" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L34" s="98"/>
+      <c r="M34" s="98"/>
+      <c r="N34" s="98"/>
+      <c r="O34" s="98"/>
+      <c r="P34" s="98"/>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="25"/>
       <c r="B35" s="4"/>
       <c r="C35" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D35" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E35" s="152" t="s">
-        <v>72</v>
-      </c>
-      <c r="F35" s="119"/>
-      <c r="G35" s="119"/>
-      <c r="H35" s="119"/>
-      <c r="I35" s="119"/>
-      <c r="J35" s="127"/>
+      <c r="D35" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E35" s="140"/>
+      <c r="F35" s="125"/>
+      <c r="G35" s="125"/>
+      <c r="H35" s="125"/>
+      <c r="I35" s="125"/>
+      <c r="J35" s="134"/>
       <c r="K35" s="25"/>
-      <c r="L35" s="99"/>
-      <c r="M35" s="99"/>
-      <c r="N35" s="99"/>
-      <c r="O35" s="99"/>
-      <c r="P35" s="99"/>
-    </row>
-    <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L35" s="98"/>
+      <c r="M35" s="98"/>
+      <c r="N35" s="98"/>
+      <c r="O35" s="98"/>
+      <c r="P35" s="98"/>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="25"/>
       <c r="B36" s="4"/>
       <c r="C36" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E36" s="153" t="s">
-        <v>37</v>
-      </c>
-      <c r="F36" s="119"/>
-      <c r="G36" s="119"/>
-      <c r="H36" s="119"/>
-      <c r="I36" s="119"/>
-      <c r="J36" s="127"/>
+        <v>35</v>
+      </c>
+      <c r="E36" s="140"/>
+      <c r="F36" s="125"/>
+      <c r="G36" s="125"/>
+      <c r="H36" s="125"/>
+      <c r="I36" s="125"/>
+      <c r="J36" s="134"/>
       <c r="K36" s="25"/>
-      <c r="L36" s="99"/>
-      <c r="M36" s="99"/>
-      <c r="N36" s="99"/>
-      <c r="O36" s="99"/>
-      <c r="P36" s="99"/>
+      <c r="L36" s="98"/>
+      <c r="M36" s="98"/>
+      <c r="N36" s="98"/>
+      <c r="O36" s="98"/>
+      <c r="P36" s="98"/>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="25"/>
@@ -3063,540 +3059,496 @@
       <c r="C37" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D37" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E37" s="153"/>
-      <c r="F37" s="119"/>
-      <c r="G37" s="119"/>
-      <c r="H37" s="119"/>
-      <c r="I37" s="119"/>
-      <c r="J37" s="127"/>
+      <c r="D37" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E37" s="140"/>
+      <c r="F37" s="125"/>
+      <c r="G37" s="125"/>
+      <c r="H37" s="125"/>
+      <c r="I37" s="125"/>
+      <c r="J37" s="134"/>
       <c r="K37" s="25"/>
-      <c r="L37" s="99"/>
-      <c r="M37" s="99"/>
-      <c r="N37" s="99"/>
-      <c r="O37" s="99"/>
-      <c r="P37" s="99"/>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L37" s="98"/>
+      <c r="M37" s="98"/>
+      <c r="N37" s="98"/>
+      <c r="O37" s="98"/>
+      <c r="P37" s="98"/>
+    </row>
+    <row r="38" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="25"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E38" s="153"/>
-      <c r="F38" s="119"/>
-      <c r="G38" s="119"/>
-      <c r="H38" s="119"/>
-      <c r="I38" s="119"/>
-      <c r="J38" s="127"/>
+      <c r="B38" s="48" t="s">
+        <v>58</v>
+      </c>
+      <c r="C38" s="49" t="s">
+        <v>41</v>
+      </c>
+      <c r="D38" s="25"/>
+      <c r="E38" s="113" t="s">
+        <v>42</v>
+      </c>
+      <c r="F38" s="124"/>
+      <c r="G38" s="124"/>
+      <c r="H38" s="124"/>
+      <c r="I38" s="124"/>
+      <c r="J38" s="106" t="s">
+        <v>133</v>
+      </c>
       <c r="K38" s="25"/>
-      <c r="L38" s="99"/>
-      <c r="M38" s="99"/>
-      <c r="N38" s="99"/>
-      <c r="O38" s="99"/>
-      <c r="P38" s="99"/>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L38" s="98"/>
+      <c r="M38" s="98"/>
+      <c r="N38" s="98"/>
+      <c r="O38" s="98"/>
+      <c r="P38" s="98"/>
+    </row>
+    <row r="39" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="25"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E39" s="153"/>
-      <c r="F39" s="119"/>
-      <c r="G39" s="119"/>
-      <c r="H39" s="119"/>
-      <c r="I39" s="119"/>
-      <c r="J39" s="127"/>
+      <c r="B39" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D39" s="3"/>
+      <c r="E39" s="114" t="s">
+        <v>62</v>
+      </c>
+      <c r="F39" s="97" t="s">
+        <v>66</v>
+      </c>
+      <c r="G39" s="141" t="s">
+        <v>68</v>
+      </c>
+      <c r="H39" s="141"/>
+      <c r="I39" s="97" t="s">
+        <v>67</v>
+      </c>
+      <c r="J39" s="107"/>
       <c r="K39" s="25"/>
-      <c r="L39" s="99"/>
-      <c r="M39" s="99"/>
-      <c r="N39" s="99"/>
-      <c r="O39" s="99"/>
-      <c r="P39" s="99"/>
-    </row>
-    <row r="40" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L39" s="98"/>
+      <c r="M39" s="98"/>
+      <c r="N39" s="98"/>
+      <c r="O39" s="98"/>
+      <c r="P39" s="98"/>
+    </row>
+    <row r="40" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="25"/>
-      <c r="B40" s="49" t="s">
+      <c r="B40" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C40" s="50" t="s">
-        <v>41</v>
-      </c>
-      <c r="D40" s="25"/>
-      <c r="E40" s="151" t="s">
-        <v>42</v>
-      </c>
-      <c r="F40" s="118"/>
-      <c r="G40" s="118"/>
-      <c r="H40" s="118"/>
-      <c r="I40" s="118"/>
-      <c r="J40" s="107" t="s">
-        <v>134</v>
-      </c>
+      <c r="C40" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D40" s="3"/>
+      <c r="E40" s="114" t="s">
+        <v>63</v>
+      </c>
+      <c r="F40" s="128"/>
+      <c r="G40" s="128"/>
+      <c r="H40" s="128"/>
+      <c r="I40" s="128"/>
+      <c r="J40" s="107"/>
       <c r="K40" s="25"/>
-      <c r="L40" s="99"/>
-      <c r="M40" s="99"/>
-      <c r="N40" s="99"/>
-      <c r="O40" s="99"/>
-      <c r="P40" s="99"/>
-    </row>
-    <row r="41" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L40" s="98"/>
+      <c r="M40" s="98"/>
+      <c r="N40" s="98"/>
+      <c r="O40" s="98"/>
+      <c r="P40" s="98"/>
+    </row>
+    <row r="41" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="25"/>
       <c r="B41" s="1" t="s">
         <v>58</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="D41" s="3"/>
-      <c r="E41" s="152" t="s">
-        <v>62</v>
-      </c>
-      <c r="F41" s="98" t="s">
+      <c r="E41" s="114" t="s">
+        <v>64</v>
+      </c>
+      <c r="F41" s="128"/>
+      <c r="G41" s="128"/>
+      <c r="H41" s="128"/>
+      <c r="I41" s="128"/>
+      <c r="J41" s="107"/>
+      <c r="K41" s="25"/>
+      <c r="L41" s="98"/>
+      <c r="M41" s="98"/>
+      <c r="N41" s="98"/>
+      <c r="O41" s="98"/>
+      <c r="P41" s="98"/>
+    </row>
+    <row r="42" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="25"/>
+      <c r="B42" s="147" t="s">
+        <v>58</v>
+      </c>
+      <c r="C42" s="148" t="s">
+        <v>73</v>
+      </c>
+      <c r="D42" s="148"/>
+      <c r="E42" s="149" t="s">
+        <v>74</v>
+      </c>
+      <c r="F42" s="95" t="s">
         <v>66</v>
       </c>
-      <c r="G41" s="132" t="s">
+      <c r="G42" s="139" t="s">
         <v>68</v>
       </c>
-      <c r="H41" s="132"/>
-      <c r="I41" s="98" t="s">
+      <c r="H42" s="139"/>
+      <c r="I42" s="95" t="s">
         <v>67</v>
       </c>
-      <c r="J41" s="108"/>
-      <c r="K41" s="25"/>
-      <c r="L41" s="99"/>
-      <c r="M41" s="99"/>
-      <c r="N41" s="99"/>
-      <c r="O41" s="99"/>
-      <c r="P41" s="99"/>
-    </row>
-    <row r="42" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="25"/>
-      <c r="B42" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D42" s="3"/>
-      <c r="E42" s="152" t="s">
-        <v>63</v>
-      </c>
-      <c r="F42" s="120"/>
-      <c r="G42" s="120"/>
-      <c r="H42" s="120"/>
-      <c r="I42" s="120"/>
-      <c r="J42" s="108"/>
+      <c r="J42" s="136"/>
       <c r="K42" s="25"/>
-      <c r="L42" s="99"/>
-      <c r="M42" s="99"/>
-      <c r="N42" s="99"/>
-      <c r="O42" s="99"/>
-      <c r="P42" s="99"/>
+      <c r="L42" s="98"/>
+      <c r="M42" s="98"/>
+      <c r="N42" s="98"/>
+      <c r="O42" s="98"/>
+      <c r="P42" s="98"/>
     </row>
     <row r="43" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="25"/>
-      <c r="B43" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D43" s="3"/>
-      <c r="E43" s="152" t="s">
-        <v>64</v>
-      </c>
-      <c r="F43" s="120"/>
-      <c r="G43" s="120"/>
-      <c r="H43" s="120"/>
-      <c r="I43" s="120"/>
-      <c r="J43" s="108"/>
+      <c r="B43" s="147"/>
+      <c r="C43" s="137"/>
+      <c r="D43" s="137"/>
+      <c r="E43" s="149"/>
+      <c r="F43" s="128"/>
+      <c r="G43" s="128"/>
+      <c r="H43" s="128"/>
+      <c r="I43" s="128"/>
+      <c r="J43" s="136"/>
       <c r="K43" s="25"/>
-      <c r="L43" s="99"/>
-      <c r="M43" s="99"/>
-      <c r="N43" s="99"/>
-      <c r="O43" s="99"/>
-      <c r="P43" s="99"/>
+      <c r="L43" s="98"/>
+      <c r="M43" s="98"/>
+      <c r="N43" s="98"/>
+      <c r="O43" s="98"/>
+      <c r="P43" s="98"/>
     </row>
     <row r="44" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="25"/>
-      <c r="B44" s="128" t="s">
+      <c r="B44" s="142" t="s">
         <v>58</v>
       </c>
-      <c r="C44" s="129" t="s">
-        <v>73</v>
-      </c>
-      <c r="D44" s="129"/>
-      <c r="E44" s="154" t="s">
-        <v>74</v>
-      </c>
-      <c r="F44" s="96" t="s">
+      <c r="C44" s="143" t="s">
+        <v>61</v>
+      </c>
+      <c r="D44" s="143"/>
+      <c r="E44" s="140" t="s">
+        <v>135</v>
+      </c>
+      <c r="F44" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="G44" s="122" t="s">
+      <c r="G44" s="129" t="s">
         <v>68</v>
       </c>
-      <c r="H44" s="122"/>
-      <c r="I44" s="96" t="s">
+      <c r="H44" s="129"/>
+      <c r="I44" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="J44" s="130"/>
+      <c r="J44" s="135"/>
       <c r="K44" s="25"/>
-      <c r="L44" s="99"/>
-      <c r="M44" s="99"/>
-      <c r="N44" s="99"/>
-      <c r="O44" s="99"/>
-      <c r="P44" s="99"/>
-    </row>
-    <row r="45" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L44" s="98"/>
+      <c r="M44" s="98"/>
+      <c r="N44" s="98"/>
+      <c r="O44" s="98"/>
+      <c r="P44" s="98"/>
+    </row>
+    <row r="45" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="25"/>
-      <c r="B45" s="128"/>
-      <c r="C45" s="131"/>
-      <c r="D45" s="131"/>
-      <c r="E45" s="154"/>
-      <c r="F45" s="120"/>
-      <c r="G45" s="120"/>
-      <c r="H45" s="120"/>
-      <c r="I45" s="120"/>
-      <c r="J45" s="130"/>
+      <c r="B45" s="142"/>
+      <c r="C45" s="144"/>
+      <c r="D45" s="144"/>
+      <c r="E45" s="140"/>
+      <c r="F45" s="145"/>
+      <c r="G45" s="145"/>
+      <c r="H45" s="146"/>
+      <c r="I45" s="146"/>
+      <c r="J45" s="135"/>
       <c r="K45" s="25"/>
-      <c r="L45" s="99"/>
-      <c r="M45" s="99"/>
-      <c r="N45" s="99"/>
-      <c r="O45" s="99"/>
-      <c r="P45" s="99"/>
-    </row>
-    <row r="46" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="25"/>
-      <c r="B46" s="133" t="s">
+      <c r="L45" s="98"/>
+      <c r="M45" s="98"/>
+      <c r="N45" s="98"/>
+      <c r="O45" s="98"/>
+      <c r="P45" s="98"/>
+    </row>
+    <row r="46" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="A46" s="98"/>
+      <c r="B46" s="150" t="s">
         <v>58</v>
       </c>
-      <c r="C46" s="134" t="s">
-        <v>61</v>
-      </c>
-      <c r="D46" s="134"/>
-      <c r="E46" s="153" t="s">
-        <v>136</v>
-      </c>
-      <c r="F46" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="G46" s="121" t="s">
-        <v>68</v>
-      </c>
-      <c r="H46" s="121"/>
-      <c r="I46" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="J46" s="135"/>
-      <c r="K46" s="25"/>
-      <c r="L46" s="99"/>
-      <c r="M46" s="99"/>
-      <c r="N46" s="99"/>
-      <c r="O46" s="99"/>
-      <c r="P46" s="99"/>
-    </row>
-    <row r="47" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="25"/>
-      <c r="B47" s="133"/>
-      <c r="C47" s="136"/>
-      <c r="D47" s="136"/>
-      <c r="E47" s="153"/>
-      <c r="F47" s="137"/>
-      <c r="G47" s="137"/>
-      <c r="H47" s="138"/>
-      <c r="I47" s="138"/>
-      <c r="J47" s="135"/>
-      <c r="K47" s="25"/>
-      <c r="L47" s="99"/>
-      <c r="M47" s="99"/>
-      <c r="N47" s="99"/>
-      <c r="O47" s="99"/>
-      <c r="P47" s="99"/>
-    </row>
-    <row r="48" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A48" s="99"/>
-      <c r="B48" s="139" t="s">
+      <c r="C46" s="151" t="s">
+        <v>104</v>
+      </c>
+      <c r="D46" s="151"/>
+      <c r="E46" s="115" t="s">
+        <v>125</v>
+      </c>
+      <c r="F46" s="152"/>
+      <c r="G46" s="152"/>
+      <c r="H46" s="152"/>
+      <c r="I46" s="152"/>
+      <c r="J46" s="153" t="s">
+        <v>134</v>
+      </c>
+      <c r="K46" s="98"/>
+      <c r="L46" s="98"/>
+      <c r="M46" s="98"/>
+      <c r="N46" s="98"/>
+      <c r="O46" s="98"/>
+      <c r="P46" s="98"/>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" s="98"/>
+      <c r="B47" s="150"/>
+      <c r="C47" s="155"/>
+      <c r="D47" s="155"/>
+      <c r="E47" s="115" t="s">
+        <v>126</v>
+      </c>
+      <c r="F47" s="152"/>
+      <c r="G47" s="152"/>
+      <c r="H47" s="152"/>
+      <c r="I47" s="152"/>
+      <c r="J47" s="154"/>
+      <c r="K47" s="98"/>
+      <c r="L47" s="98"/>
+      <c r="M47" s="98"/>
+      <c r="N47" s="98"/>
+      <c r="O47" s="98"/>
+      <c r="P47" s="98"/>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A48" s="98"/>
+      <c r="B48" s="150"/>
+      <c r="C48" s="155"/>
+      <c r="D48" s="155"/>
+      <c r="E48" s="115" t="s">
+        <v>127</v>
+      </c>
+      <c r="F48" s="152"/>
+      <c r="G48" s="152"/>
+      <c r="H48" s="152"/>
+      <c r="I48" s="152"/>
+      <c r="J48" s="154"/>
+      <c r="K48" s="98"/>
+      <c r="L48" s="98"/>
+      <c r="M48" s="98"/>
+      <c r="N48" s="98"/>
+      <c r="O48" s="98"/>
+      <c r="P48" s="98"/>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A49" s="98"/>
+      <c r="B49" s="150"/>
+      <c r="C49" s="155"/>
+      <c r="D49" s="155"/>
+      <c r="E49" s="115" t="s">
+        <v>128</v>
+      </c>
+      <c r="F49" s="152"/>
+      <c r="G49" s="152"/>
+      <c r="H49" s="152"/>
+      <c r="I49" s="152"/>
+      <c r="J49" s="154"/>
+      <c r="K49" s="98"/>
+      <c r="L49" s="98"/>
+      <c r="M49" s="98"/>
+      <c r="N49" s="98"/>
+      <c r="O49" s="98"/>
+      <c r="P49" s="98"/>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A50" s="25"/>
+      <c r="B50" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C48" s="140" t="s">
-        <v>105</v>
-      </c>
-      <c r="D48" s="140"/>
-      <c r="E48" s="155" t="s">
-        <v>126</v>
-      </c>
-      <c r="F48" s="141"/>
-      <c r="G48" s="141"/>
-      <c r="H48" s="141"/>
-      <c r="I48" s="141"/>
-      <c r="J48" s="142" t="s">
-        <v>135</v>
-      </c>
-      <c r="K48" s="99"/>
-      <c r="L48" s="99"/>
-      <c r="M48" s="99"/>
-      <c r="N48" s="99"/>
-      <c r="O48" s="99"/>
-      <c r="P48" s="99"/>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A49" s="99"/>
-      <c r="B49" s="139"/>
-      <c r="C49" s="144"/>
-      <c r="D49" s="144"/>
-      <c r="E49" s="155" t="s">
-        <v>127</v>
-      </c>
-      <c r="F49" s="141"/>
-      <c r="G49" s="141"/>
-      <c r="H49" s="141"/>
-      <c r="I49" s="141"/>
-      <c r="J49" s="143"/>
-      <c r="K49" s="99"/>
-      <c r="L49" s="99"/>
-      <c r="M49" s="99"/>
-      <c r="N49" s="99"/>
-      <c r="O49" s="99"/>
-      <c r="P49" s="99"/>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A50" s="99"/>
-      <c r="B50" s="139"/>
-      <c r="C50" s="144"/>
-      <c r="D50" s="144"/>
-      <c r="E50" s="155" t="s">
-        <v>128</v>
-      </c>
-      <c r="F50" s="141"/>
-      <c r="G50" s="141"/>
-      <c r="H50" s="141"/>
-      <c r="I50" s="141"/>
-      <c r="J50" s="143"/>
-      <c r="K50" s="99"/>
-      <c r="L50" s="99"/>
-      <c r="M50" s="99"/>
-      <c r="N50" s="99"/>
-      <c r="O50" s="99"/>
-      <c r="P50" s="99"/>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A51" s="99"/>
-      <c r="B51" s="139"/>
-      <c r="C51" s="144"/>
-      <c r="D51" s="144"/>
-      <c r="E51" s="155" t="s">
-        <v>129</v>
-      </c>
-      <c r="F51" s="141"/>
-      <c r="G51" s="141"/>
-      <c r="H51" s="141"/>
-      <c r="I51" s="141"/>
-      <c r="J51" s="143"/>
-      <c r="K51" s="99"/>
-      <c r="L51" s="99"/>
-      <c r="M51" s="99"/>
-      <c r="N51" s="99"/>
-      <c r="O51" s="99"/>
-      <c r="P51" s="99"/>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="C50" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D50" s="3"/>
+      <c r="E50" s="114" t="s">
+        <v>47</v>
+      </c>
+      <c r="F50" s="138"/>
+      <c r="G50" s="138"/>
+      <c r="H50" s="138"/>
+      <c r="I50" s="138"/>
+      <c r="J50" s="107"/>
+      <c r="K50" s="25"/>
+      <c r="L50" s="98"/>
+      <c r="M50" s="98"/>
+      <c r="N50" s="98"/>
+      <c r="O50" s="98"/>
+      <c r="P50" s="98"/>
+    </row>
+    <row r="51" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="25"/>
+      <c r="B51" s="48" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="D51" s="25"/>
+      <c r="E51" s="113" t="s">
+        <v>76</v>
+      </c>
+      <c r="F51" s="124"/>
+      <c r="G51" s="124"/>
+      <c r="H51" s="124"/>
+      <c r="I51" s="124"/>
+      <c r="J51" s="106" t="s">
+        <v>130</v>
+      </c>
+      <c r="K51" s="25"/>
+      <c r="L51" s="98"/>
+      <c r="M51" s="98"/>
+      <c r="N51" s="98"/>
+      <c r="O51" s="98"/>
+      <c r="P51" s="98"/>
+    </row>
+    <row r="52" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="25"/>
       <c r="B52" s="1" t="s">
         <v>58</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D52" s="3"/>
-      <c r="E52" s="152" t="s">
-        <v>47</v>
-      </c>
-      <c r="F52" s="145"/>
-      <c r="G52" s="145"/>
-      <c r="H52" s="145"/>
-      <c r="I52" s="145"/>
-      <c r="J52" s="108"/>
+      <c r="E52" s="114" t="s">
+        <v>51</v>
+      </c>
+      <c r="F52" s="125"/>
+      <c r="G52" s="125"/>
+      <c r="H52" s="125"/>
+      <c r="I52" s="125"/>
+      <c r="J52" s="108" t="s">
+        <v>131</v>
+      </c>
       <c r="K52" s="25"/>
-      <c r="L52" s="99"/>
-      <c r="M52" s="99"/>
-      <c r="N52" s="99"/>
-      <c r="O52" s="99"/>
-      <c r="P52" s="99"/>
-    </row>
-    <row r="53" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L52" s="98"/>
+      <c r="M52" s="98"/>
+      <c r="N52" s="98"/>
+      <c r="O52" s="98"/>
+      <c r="P52" s="98"/>
+    </row>
+    <row r="53" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="25"/>
-      <c r="B53" s="49" t="s">
+      <c r="B53" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="C53" s="50" t="s">
-        <v>49</v>
-      </c>
-      <c r="D53" s="25"/>
-      <c r="E53" s="151" t="s">
-        <v>76</v>
-      </c>
-      <c r="F53" s="118"/>
-      <c r="G53" s="118"/>
-      <c r="H53" s="118"/>
-      <c r="I53" s="118"/>
-      <c r="J53" s="107" t="s">
-        <v>131</v>
+      <c r="C53" s="117" t="s">
+        <v>52</v>
+      </c>
+      <c r="D53" s="117"/>
+      <c r="E53" s="113" t="s">
+        <v>75</v>
+      </c>
+      <c r="F53" s="124"/>
+      <c r="G53" s="124"/>
+      <c r="H53" s="124"/>
+      <c r="I53" s="124"/>
+      <c r="J53" s="106" t="s">
+        <v>132</v>
       </c>
       <c r="K53" s="25"/>
-      <c r="L53" s="99"/>
-      <c r="M53" s="99"/>
-      <c r="N53" s="99"/>
-      <c r="O53" s="99"/>
-      <c r="P53" s="99"/>
-    </row>
-    <row r="54" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L53" s="98"/>
+      <c r="M53" s="98"/>
+      <c r="N53" s="98"/>
+      <c r="O53" s="98"/>
+      <c r="P53" s="98"/>
+    </row>
+    <row r="54" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="25"/>
-      <c r="B54" s="1" t="s">
+      <c r="B54" s="99" t="s">
         <v>58</v>
       </c>
-      <c r="C54" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D54" s="3"/>
-      <c r="E54" s="152" t="s">
-        <v>51</v>
-      </c>
-      <c r="F54" s="119"/>
-      <c r="G54" s="119"/>
-      <c r="H54" s="119"/>
-      <c r="I54" s="119"/>
-      <c r="J54" s="109" t="s">
-        <v>132</v>
-      </c>
+      <c r="C54" s="100" t="s">
+        <v>53</v>
+      </c>
+      <c r="D54" s="101"/>
+      <c r="E54" s="116" t="s">
+        <v>54</v>
+      </c>
+      <c r="F54" s="102"/>
+      <c r="G54" s="102"/>
+      <c r="H54" s="102"/>
+      <c r="I54" s="102"/>
+      <c r="J54" s="109"/>
       <c r="K54" s="25"/>
-      <c r="L54" s="99"/>
-      <c r="M54" s="99"/>
-      <c r="N54" s="99"/>
-      <c r="O54" s="99"/>
-      <c r="P54" s="99"/>
-    </row>
-    <row r="55" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L54" s="98"/>
+      <c r="M54" s="98"/>
+      <c r="N54" s="98"/>
+      <c r="O54" s="98"/>
+      <c r="P54" s="98"/>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="25"/>
-      <c r="B55" s="49" t="s">
-        <v>58</v>
-      </c>
-      <c r="C55" s="111" t="s">
-        <v>52</v>
-      </c>
-      <c r="D55" s="111"/>
-      <c r="E55" s="151" t="s">
-        <v>75</v>
-      </c>
-      <c r="F55" s="118"/>
-      <c r="G55" s="118"/>
-      <c r="H55" s="118"/>
-      <c r="I55" s="118"/>
-      <c r="J55" s="107" t="s">
-        <v>133</v>
-      </c>
+      <c r="B55" s="25"/>
+      <c r="C55" s="25"/>
+      <c r="D55" s="25"/>
+      <c r="E55" s="29"/>
+      <c r="F55" s="31"/>
+      <c r="G55" s="31"/>
+      <c r="H55" s="31"/>
+      <c r="I55" s="31"/>
+      <c r="J55" s="25"/>
       <c r="K55" s="25"/>
-      <c r="L55" s="99"/>
-      <c r="M55" s="99"/>
-      <c r="N55" s="99"/>
-      <c r="O55" s="99"/>
-      <c r="P55" s="99"/>
-    </row>
-    <row r="56" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="25"/>
-      <c r="B56" s="100" t="s">
-        <v>58</v>
-      </c>
-      <c r="C56" s="101" t="s">
-        <v>53</v>
-      </c>
-      <c r="D56" s="102"/>
-      <c r="E56" s="156" t="s">
-        <v>54</v>
-      </c>
-      <c r="F56" s="103"/>
-      <c r="G56" s="103"/>
-      <c r="H56" s="103"/>
-      <c r="I56" s="103"/>
-      <c r="J56" s="110"/>
-      <c r="K56" s="25"/>
-      <c r="L56" s="99"/>
-      <c r="M56" s="99"/>
-      <c r="N56" s="99"/>
-      <c r="O56" s="99"/>
-      <c r="P56" s="99"/>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A57" s="25"/>
-      <c r="B57" s="25"/>
-      <c r="C57" s="25"/>
-      <c r="D57" s="25"/>
-      <c r="E57" s="29"/>
-      <c r="F57" s="31"/>
-      <c r="G57" s="31"/>
-      <c r="H57" s="31"/>
-      <c r="I57" s="31"/>
-      <c r="J57" s="25"/>
-      <c r="K57" s="25"/>
-      <c r="L57" s="99"/>
-      <c r="M57" s="99"/>
-      <c r="N57" s="99"/>
-      <c r="O57" s="99"/>
-      <c r="P57" s="99"/>
+      <c r="L55" s="98"/>
+      <c r="M55" s="98"/>
+      <c r="N55" s="98"/>
+      <c r="O55" s="98"/>
+      <c r="P55" s="98"/>
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="B48:B51"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="F48:I51"/>
-    <mergeCell ref="J48:J51"/>
-    <mergeCell ref="C49:D51"/>
-    <mergeCell ref="E36:E39"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="J46:J49"/>
+    <mergeCell ref="C47:D49"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:E43"/>
+    <mergeCell ref="B46:B49"/>
     <mergeCell ref="C46:D46"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="H47:I47"/>
     <mergeCell ref="B44:B45"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="E44:E45"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="F50:I50"/>
+    <mergeCell ref="F51:I51"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="F46:I49"/>
+    <mergeCell ref="J19:J26"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="J32:J37"/>
     <mergeCell ref="J44:J45"/>
-    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="J42:J43"/>
+    <mergeCell ref="C53:D53"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="F11:I18"/>
+    <mergeCell ref="F19:I26"/>
+    <mergeCell ref="F27:I28"/>
+    <mergeCell ref="F29:I30"/>
+    <mergeCell ref="F31:I31"/>
+    <mergeCell ref="F32:I37"/>
+    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F40:I41"/>
+    <mergeCell ref="F43:I43"/>
+    <mergeCell ref="F53:I53"/>
     <mergeCell ref="F52:I52"/>
-    <mergeCell ref="F53:I53"/>
     <mergeCell ref="G44:H44"/>
-    <mergeCell ref="J21:J28"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J34:J39"/>
-    <mergeCell ref="J46:J47"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="F12:I12"/>
-    <mergeCell ref="F13:I20"/>
-    <mergeCell ref="F21:I28"/>
-    <mergeCell ref="F29:I30"/>
-    <mergeCell ref="F31:I32"/>
-    <mergeCell ref="F33:I33"/>
-    <mergeCell ref="F34:I39"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F42:I43"/>
-    <mergeCell ref="F45:I45"/>
-    <mergeCell ref="F55:I55"/>
-    <mergeCell ref="F54:I54"/>
-    <mergeCell ref="G46:H46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3604,228 +3556,228 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A44"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="51" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="52" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="53" t="s">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="53" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="54" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="54" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="55" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="55" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="56" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="56" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="57" t="s">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="57" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="58" t="s">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="58" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="59" t="s">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="59" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="60" t="s">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="60" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="61" t="s">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="61" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="62" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="62" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="63" t="s">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="63" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="64" t="s">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="64" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="65" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="65" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="66" t="s">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="66" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="67" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="67" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="68" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="68" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="69" t="s">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="69" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="70" t="s">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="70" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="71" t="s">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="71" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="72" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="72" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="73" t="s">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="73" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="74" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="74" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="75" t="s">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="75" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="76" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="76" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="77" t="s">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="77" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" s="78" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="78" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" s="79" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="79" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" s="80" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="80" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" s="81" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="81" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" s="82" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="82" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" s="83" t="s">
+    <row r="33" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="83" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="84" t="s">
+    <row r="34" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="84" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="34" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="85" t="s">
+    <row r="35" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="85" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="35" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="86" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="86" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" s="87" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="87" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" s="88" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="88" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" s="89" t="s">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="89" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" s="90" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="90" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" s="91" t="s">
+    <row r="41" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="91" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="41" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="92" t="s">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="92" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" s="93" t="s">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="93" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" s="94" t="s">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="94" t="s">
         <v>124</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" s="95" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>